<commit_message>
Update app logic, pipeline filter, and OCR engine safely
</commit_message>
<xml_diff>
--- a/data/goods_records.xlsx
+++ b/data/goods_records.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -583,6 +583,111 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
+        <is>
+          <t>In Transit</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>114082</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>RATHI</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>S.S.T. LOGISTIC</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>14-08-2026</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>In Transit</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>KRJKT04754</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>OKK</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>SHIV SHANKAR</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>01-09-2026</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>10</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>In Transit</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>KRJKT04612</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>OOK</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>SHIV SHANKAR</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>30-08-2026</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
         <is>
           <t>In Transit</t>
         </is>

</xml_diff>

<commit_message>
Connect repository and update core app logic
</commit_message>
<xml_diff>
--- a/data/goods_records.xlsx
+++ b/data/goods_records.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,224 +472,6 @@
       <c r="I1" s="1" t="inlineStr">
         <is>
           <t>status</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>KRJKT04677</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Riddi</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>sst</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>31-08-2026</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Received</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>KRJKT04672</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Riddi</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>SHIV SHANKAR</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>31-08-2026</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Received</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>KSHPRO0411</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Yamuna</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>SHIV SHANKAR</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>31-08-2026</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>22</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>In Transit</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>114082</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>RATHI</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>S.S.T. LOGISTIC</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>14-08-2026</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>In Transit</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>KRJKT04754</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>OKK</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>SHIV SHANKAR</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>01-09-2026</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>10</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>In Transit</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>KRJKT04612</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>OOK</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>SHIV SHANKAR</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>30-08-2026</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>In Transit</t>
         </is>
       </c>
     </row>

</xml_diff>